<commit_message>
cambio global main en do file 1 y guardo un recuperado
</commit_message>
<xml_diff>
--- a/Procesamiento de datos/Output/tabla_balance_bes_subset.xlsx
+++ b/Procesamiento de datos/Output/tabla_balance_bes_subset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/florenciaruiz/Library/Mobile Documents/com~apple~CloudDocs/RA Maria/Tres de Febrero/Tres_de_Febrero/Procesamiento de datos/Output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88456B3-35EA-714A-BECF-FCC7C1DA6737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364017ED-CEFE-B04B-BD6B-6FA8C4DE1E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2980" yWindow="-20280" windowWidth="25800" windowHeight="17620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -572,6 +572,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">

</xml_diff>